<commit_message>
docs: cap nhat file ket qua test case
</commit_message>
<xml_diff>
--- a/Extra/Phân công.xlsx
+++ b/Extra/Phân công.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/07c1b08ee16acfbd/Tài liệu/UTH (ws)/LapTrinhMang/012012301310_Group04_UDM09/Extra/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\012012301310_Group04_UDM09\Extra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3B14E54-2BBE-4D7A-9844-D4EB0D2C286D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E90C2D68-8934-4DFD-95E2-6FA8CF8F7186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -93,9 +93,6 @@
     <t>052206003938</t>
   </si>
   <si>
-    <t>Nguyễn Phan Hoài Bình</t>
-  </si>
-  <si>
     <t>Giao thức (Protocol) &amp; Quản lý Truyền tải File</t>
   </si>
   <si>
@@ -202,6 +199,9 @@
   </si>
   <si>
     <t xml:space="preserve">Trần Thị Thanh Thơ </t>
+  </si>
+  <si>
+    <t>Nguyễn Phan Hoài Bin</t>
   </si>
 </sst>
 </file>
@@ -693,68 +693,68 @@
         <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="C5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="F5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>53</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="218.4" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -775,57 +775,57 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="8" t="s">
         <v>39</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>